<commit_message>
Free templates: Legal desk fixes and design round 1 fixes (still drafts)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0122otiWoh8gJECjGVg2FuAQ
</commit_message>
<xml_diff>
--- a/docs/downloads/job-estimate-template.xlsx
+++ b/docs/downloads/job-estimate-template.xlsx
@@ -21,8 +21,8 @@
     <definedName name="TaxRate">'Estimate'!$J$19</definedName>
     <definedName name="DepositRate">'Estimate'!$J$20</definedName>
     <definedName name="PaymentTerms">'Estimate'!$D$40</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Start Here'!$A$1:$G$45</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Estimate'!$A$1:$L$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Start Here'!$A$1:$G$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Estimate'!$A$1:$L$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Terms'!$A$1:$G$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -206,7 +206,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -345,6 +345,56 @@
       </bottom>
     </border>
     <border>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E3C978"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E3C978"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E3C978"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E3C978"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E3C978"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E3C978"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E3C978"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E3C978"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E3C978"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thin">
         <color rgb="001D2433"/>
       </top>
@@ -426,7 +476,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -478,21 +528,21 @@
     <xf numFmtId="168" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="15" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="17" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -502,9 +552,9 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -563,6 +613,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="15" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
       <protection locked="0" hidden="0"/>
@@ -577,14 +628,21 @@
     <xf numFmtId="167" fontId="6" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -965,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z84"/>
+  <dimension ref="A1:Z85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2225,7 +2283,7 @@
       <c r="Y35" s="1" t="n"/>
       <c r="Z35" s="1" t="n"/>
     </row>
-    <row r="36" ht="37.6" customHeight="1">
+    <row r="36" ht="63.2" customHeight="1">
       <c r="A36" s="1" t="n"/>
       <c r="B36" s="10" t="n"/>
       <c r="C36" s="14" t="inlineStr">
@@ -2237,7 +2295,7 @@
               <color rgb="001D2433"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Pricing each line. </t>
+            <t xml:space="preserve">Deposits and cancelling. </t>
           </r>
           <r>
             <rPr>
@@ -2245,7 +2303,7 @@
               <color rgb="001D2433"/>
               <sz val="10"/>
             </rPr>
-            <t>The free calculators at proofnotfluff.com price a clean, a lawn visit or a pressure washing job from your own costs and time. The Terms tab links them.</t>
+            <t>Rules on deposits, cancelling and the wording of signed estimates vary by state and city, especially for work sold at the customer's home. This template doesn't say what any law requires. Have a local attorney check your deposit, payment and cancellation terms before you use them with clients.</t>
           </r>
         </is>
       </c>
@@ -2285,7 +2343,7 @@
               <color rgb="001D2433"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Google Sheets. </t>
+            <t xml:space="preserve">Pricing each line. </t>
           </r>
           <r>
             <rPr>
@@ -2293,7 +2351,7 @@
               <color rgb="001D2433"/>
               <sz val="10"/>
             </rPr>
-            <t>Upload the .xlsx to Google Drive, open it, then File, Save as Google Sheets. No macros, no add-ons.</t>
+            <t>The free calculators at proofnotfluff.com price a clean, a lawn visit or a pressure washing job from your own costs and time. The Terms tab links them.</t>
           </r>
         </is>
       </c>
@@ -2321,13 +2379,33 @@
       <c r="Y37" s="1" t="n"/>
       <c r="Z37" s="1" t="n"/>
     </row>
-    <row r="38" ht="12" customHeight="1">
+    <row r="38" ht="37.6" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="16" t="n"/>
-      <c r="D38" s="16" t="n"/>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="17" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="001D2433"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">Google Sheets. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="001D2433"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Upload the .xlsx to Google Drive, open it, then File, Save as Google Sheets. No macros, no add-ons.</t>
+          </r>
+        </is>
+      </c>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="13" t="n"/>
       <c r="G38" s="1" t="n"/>
       <c r="H38" s="1" t="n"/>
       <c r="I38" s="1" t="n"/>
@@ -2349,13 +2427,13 @@
       <c r="Y38" s="1" t="n"/>
       <c r="Z38" s="1" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" ht="12" customHeight="1">
       <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="16" t="n"/>
+      <c r="D39" s="16" t="n"/>
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="17" t="n"/>
       <c r="G39" s="1" t="n"/>
       <c r="H39" s="1" t="n"/>
       <c r="I39" s="1" t="n"/>
@@ -2377,13 +2455,13 @@
       <c r="Y39" s="1" t="n"/>
       <c r="Z39" s="1" t="n"/>
     </row>
-    <row r="40" ht="12" customHeight="1">
+    <row r="40">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="8" t="n"/>
-      <c r="E40" s="8" t="n"/>
-      <c r="F40" s="9" t="n"/>
+      <c r="B40" s="1" t="n"/>
+      <c r="C40" s="1" t="n"/>
+      <c r="D40" s="1" t="n"/>
+      <c r="E40" s="1" t="n"/>
+      <c r="F40" s="1" t="n"/>
       <c r="G40" s="1" t="n"/>
       <c r="H40" s="1" t="n"/>
       <c r="I40" s="1" t="n"/>
@@ -2405,17 +2483,13 @@
       <c r="Y40" s="1" t="n"/>
       <c r="Z40" s="1" t="n"/>
     </row>
-    <row r="41" ht="24" customHeight="1">
+    <row r="41" ht="12" customHeight="1">
       <c r="A41" s="1" t="n"/>
-      <c r="B41" s="10" t="n"/>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>Before you rely on a number</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="n"/>
-      <c r="F41" s="13" t="n"/>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="9" t="n"/>
       <c r="G41" s="1" t="n"/>
       <c r="H41" s="1" t="n"/>
       <c r="I41" s="1" t="n"/>
@@ -2437,12 +2511,12 @@
       <c r="Y41" s="1" t="n"/>
       <c r="Z41" s="1" t="n"/>
     </row>
-    <row r="42" ht="63.2" customHeight="1">
+    <row r="42" ht="24" customHeight="1">
       <c r="A42" s="1" t="n"/>
       <c r="B42" s="10" t="n"/>
-      <c r="C42" s="22" t="inlineStr">
-        <is>
-          <t>For general information and planning only. This is not legal, tax, financial, medical or other professional advice, and using it doesn't create a professional relationship. Results are estimates based on the numbers you enter. Figures were checked on October 26, 2026 and can change. See the Terms tab before you rely on anything here.</t>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Before you rely on a number</t>
         </is>
       </c>
       <c r="D42" s="12" t="n"/>
@@ -2469,12 +2543,12 @@
       <c r="Y42" s="1" t="n"/>
       <c r="Z42" s="1" t="n"/>
     </row>
-    <row r="43" ht="50.4" customHeight="1">
+    <row r="43" ht="63.2" customHeight="1">
       <c r="A43" s="1" t="n"/>
       <c r="B43" s="10" t="n"/>
       <c r="C43" s="22" t="inlineStr">
         <is>
-          <t>These are sample forms to adapt, not legal documents written for your state or business. Have a local attorney review any agreement before you use it with clients. If you collect client information, you're responsible for keeping it secure and following the privacy laws that apply to you.</t>
+          <t>For general information and planning only. This is not legal, tax, financial, medical or other professional advice, and using it doesn't create a professional relationship. Results are estimates based on the numbers you enter. Figures were checked on October 26, 2026 and can change. See the Terms tab before you rely on anything here.</t>
         </is>
       </c>
       <c r="D43" s="12" t="n"/>
@@ -2501,13 +2575,17 @@
       <c r="Y43" s="1" t="n"/>
       <c r="Z43" s="1" t="n"/>
     </row>
-    <row r="44" ht="12" customHeight="1">
+    <row r="44" ht="50.4" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="15" t="n"/>
-      <c r="C44" s="16" t="n"/>
-      <c r="D44" s="16" t="n"/>
-      <c r="E44" s="16" t="n"/>
-      <c r="F44" s="17" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>These are sample forms to adapt, not legal documents written for your state or business. Have a local attorney review any agreement before you use it with clients. If you collect client information, you're responsible for keeping it secure and following the privacy laws that apply to you.</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="13" t="n"/>
       <c r="G44" s="1" t="n"/>
       <c r="H44" s="1" t="n"/>
       <c r="I44" s="1" t="n"/>
@@ -2529,13 +2607,13 @@
       <c r="Y44" s="1" t="n"/>
       <c r="Z44" s="1" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" ht="12" customHeight="1">
       <c r="A45" s="1" t="n"/>
-      <c r="B45" s="1" t="n"/>
-      <c r="C45" s="1" t="n"/>
-      <c r="D45" s="1" t="n"/>
-      <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="n"/>
+      <c r="B45" s="15" t="n"/>
+      <c r="C45" s="16" t="n"/>
+      <c r="D45" s="16" t="n"/>
+      <c r="E45" s="16" t="n"/>
+      <c r="F45" s="17" t="n"/>
       <c r="G45" s="1" t="n"/>
       <c r="H45" s="1" t="n"/>
       <c r="I45" s="1" t="n"/>
@@ -3649,11 +3727,39 @@
       <c r="Y84" s="1" t="n"/>
       <c r="Z84" s="1" t="n"/>
     </row>
+    <row r="85">
+      <c r="A85" s="1" t="n"/>
+      <c r="B85" s="1" t="n"/>
+      <c r="C85" s="1" t="n"/>
+      <c r="D85" s="1" t="n"/>
+      <c r="E85" s="1" t="n"/>
+      <c r="F85" s="1" t="n"/>
+      <c r="G85" s="1" t="n"/>
+      <c r="H85" s="1" t="n"/>
+      <c r="I85" s="1" t="n"/>
+      <c r="J85" s="1" t="n"/>
+      <c r="K85" s="1" t="n"/>
+      <c r="L85" s="1" t="n"/>
+      <c r="M85" s="1" t="n"/>
+      <c r="N85" s="1" t="n"/>
+      <c r="O85" s="1" t="n"/>
+      <c r="P85" s="1" t="n"/>
+      <c r="Q85" s="1" t="n"/>
+      <c r="R85" s="1" t="n"/>
+      <c r="S85" s="1" t="n"/>
+      <c r="T85" s="1" t="n"/>
+      <c r="U85" s="1" t="n"/>
+      <c r="V85" s="1" t="n"/>
+      <c r="W85" s="1" t="n"/>
+      <c r="X85" s="1" t="n"/>
+      <c r="Y85" s="1" t="n"/>
+      <c r="Z85" s="1" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="D20:E20"/>
-    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="C44:E44"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="C12:E12"/>
@@ -3666,6 +3772,7 @@
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C38:E38"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C37:E37"/>
@@ -3703,7 +3810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z86"/>
+  <dimension ref="A1:Z87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4742,9 +4849,9 @@
           <t>2-story house, soft wash</t>
         </is>
       </c>
-      <c r="E28" s="41" t="n"/>
-      <c r="F28" s="41" t="n"/>
-      <c r="G28" s="59" t="n">
+      <c r="E28" s="59" t="n"/>
+      <c r="F28" s="59" t="n"/>
+      <c r="G28" s="60" t="n">
         <v>1</v>
       </c>
       <c r="H28" s="58" t="inlineStr">
@@ -4752,10 +4859,10 @@
           <t>job</t>
         </is>
       </c>
-      <c r="I28" s="60" t="n">
+      <c r="I28" s="61" t="n">
         <v>355</v>
       </c>
-      <c r="J28" s="61">
+      <c r="J28" s="62">
         <f>IF(OR($G28="",$I28=""),"",ROUND($G28*$I28,2))</f>
         <v/>
       </c>
@@ -4789,9 +4896,9 @@
           <t>2-car concrete, surface clean</t>
         </is>
       </c>
-      <c r="E29" s="41" t="n"/>
-      <c r="F29" s="41" t="n"/>
-      <c r="G29" s="59" t="n">
+      <c r="E29" s="59" t="n"/>
+      <c r="F29" s="59" t="n"/>
+      <c r="G29" s="60" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="58" t="inlineStr">
@@ -4799,10 +4906,10 @@
           <t>job</t>
         </is>
       </c>
-      <c r="I29" s="60" t="n">
+      <c r="I29" s="61" t="n">
         <v>200</v>
       </c>
-      <c r="J29" s="61">
+      <c r="J29" s="62">
         <f>IF(OR($G29="",$I29=""),"",ROUND($G29*$I29,2))</f>
         <v/>
       </c>
@@ -4836,9 +4943,9 @@
           <t>Face brightening, front and back</t>
         </is>
       </c>
-      <c r="E30" s="41" t="n"/>
-      <c r="F30" s="41" t="n"/>
-      <c r="G30" s="59" t="n">
+      <c r="E30" s="59" t="n"/>
+      <c r="F30" s="59" t="n"/>
+      <c r="G30" s="60" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="58" t="inlineStr">
@@ -4846,10 +4953,10 @@
           <t>job</t>
         </is>
       </c>
-      <c r="I30" s="60" t="n">
+      <c r="I30" s="61" t="n">
         <v>205</v>
       </c>
-      <c r="J30" s="61">
+      <c r="J30" s="62">
         <f>IF(OR($G30="",$I30=""),"",ROUND($G30*$I30,2))</f>
         <v/>
       </c>
@@ -4875,12 +4982,12 @@
       <c r="B31" s="10" t="n"/>
       <c r="C31" s="58" t="n"/>
       <c r="D31" s="58" t="n"/>
-      <c r="E31" s="41" t="n"/>
-      <c r="F31" s="41" t="n"/>
-      <c r="G31" s="59" t="n"/>
+      <c r="E31" s="59" t="n"/>
+      <c r="F31" s="59" t="n"/>
+      <c r="G31" s="60" t="n"/>
       <c r="H31" s="58" t="n"/>
-      <c r="I31" s="60" t="n"/>
-      <c r="J31" s="61">
+      <c r="I31" s="61" t="n"/>
+      <c r="J31" s="62">
         <f>IF(OR($G31="",$I31=""),"",ROUND($G31*$I31,2))</f>
         <v/>
       </c>
@@ -4906,12 +5013,12 @@
       <c r="B32" s="10" t="n"/>
       <c r="C32" s="58" t="n"/>
       <c r="D32" s="58" t="n"/>
-      <c r="E32" s="41" t="n"/>
-      <c r="F32" s="41" t="n"/>
-      <c r="G32" s="59" t="n"/>
+      <c r="E32" s="59" t="n"/>
+      <c r="F32" s="59" t="n"/>
+      <c r="G32" s="60" t="n"/>
       <c r="H32" s="58" t="n"/>
-      <c r="I32" s="60" t="n"/>
-      <c r="J32" s="61">
+      <c r="I32" s="61" t="n"/>
+      <c r="J32" s="62">
         <f>IF(OR($G32="",$I32=""),"",ROUND($G32*$I32,2))</f>
         <v/>
       </c>
@@ -4937,12 +5044,12 @@
       <c r="B33" s="10" t="n"/>
       <c r="C33" s="58" t="n"/>
       <c r="D33" s="58" t="n"/>
-      <c r="E33" s="41" t="n"/>
-      <c r="F33" s="41" t="n"/>
-      <c r="G33" s="59" t="n"/>
+      <c r="E33" s="59" t="n"/>
+      <c r="F33" s="59" t="n"/>
+      <c r="G33" s="60" t="n"/>
       <c r="H33" s="58" t="n"/>
-      <c r="I33" s="60" t="n"/>
-      <c r="J33" s="61">
+      <c r="I33" s="61" t="n"/>
+      <c r="J33" s="62">
         <f>IF(OR($G33="",$I33=""),"",ROUND($G33*$I33,2))</f>
         <v/>
       </c>
@@ -4968,12 +5075,12 @@
       <c r="B34" s="10" t="n"/>
       <c r="C34" s="58" t="n"/>
       <c r="D34" s="58" t="n"/>
-      <c r="E34" s="41" t="n"/>
-      <c r="F34" s="41" t="n"/>
-      <c r="G34" s="59" t="n"/>
+      <c r="E34" s="59" t="n"/>
+      <c r="F34" s="59" t="n"/>
+      <c r="G34" s="60" t="n"/>
       <c r="H34" s="58" t="n"/>
-      <c r="I34" s="60" t="n"/>
-      <c r="J34" s="61">
+      <c r="I34" s="61" t="n"/>
+      <c r="J34" s="62">
         <f>IF(OR($G34="",$I34=""),"",ROUND($G34*$I34,2))</f>
         <v/>
       </c>
@@ -4999,12 +5106,12 @@
       <c r="B35" s="10" t="n"/>
       <c r="C35" s="58" t="n"/>
       <c r="D35" s="58" t="n"/>
-      <c r="E35" s="41" t="n"/>
-      <c r="F35" s="41" t="n"/>
-      <c r="G35" s="59" t="n"/>
+      <c r="E35" s="59" t="n"/>
+      <c r="F35" s="59" t="n"/>
+      <c r="G35" s="60" t="n"/>
       <c r="H35" s="58" t="n"/>
-      <c r="I35" s="60" t="n"/>
-      <c r="J35" s="61">
+      <c r="I35" s="61" t="n"/>
+      <c r="J35" s="62">
         <f>IF(OR($G35="",$I35=""),"",ROUND($G35*$I35,2))</f>
         <v/>
       </c>
@@ -5127,7 +5234,7 @@
       </c>
       <c r="H39" s="48" t="n"/>
       <c r="I39" s="48" t="n"/>
-      <c r="J39" s="62">
+      <c r="J39" s="63">
         <f>IF(COUNT($J$28:$J$35)=0,"",SUM($J$28:$J$35))</f>
         <v/>
       </c>
@@ -5156,7 +5263,7 @@
           <t>Payment terms</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
+      <c r="D40" s="64" t="inlineStr">
         <is>
           <t>Balance due when the job is done.</t>
         </is>
@@ -5169,7 +5276,7 @@
       </c>
       <c r="H40" s="48" t="n"/>
       <c r="I40" s="48" t="n"/>
-      <c r="J40" s="62">
+      <c r="J40" s="63">
         <f>IF($J$39="","",-ROUND($J$39*N($J$18),2))</f>
         <v/>
       </c>
@@ -5193,12 +5300,8 @@
     <row r="41" ht="21" customHeight="1">
       <c r="A41" s="1" t="n"/>
       <c r="B41" s="10" t="n"/>
-      <c r="C41" s="63" t="inlineStr">
-        <is>
-          <t>To accept, sign below and return it with the deposit.</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="n"/>
+      <c r="C41" s="12" t="n"/>
+      <c r="D41" s="65" t="n"/>
       <c r="E41" s="13" t="n"/>
       <c r="F41" s="10" t="n"/>
       <c r="G41" s="47">
@@ -5207,7 +5310,7 @@
       </c>
       <c r="H41" s="48" t="n"/>
       <c r="I41" s="48" t="n"/>
-      <c r="J41" s="62">
+      <c r="J41" s="63">
         <f>IF($J$39="","",ROUND(($J$39+$J$40)*N($J$19),2))</f>
         <v/>
       </c>
@@ -5231,22 +5334,22 @@
     <row r="42" ht="21" customHeight="1">
       <c r="A42" s="1" t="n"/>
       <c r="B42" s="10" t="n"/>
-      <c r="C42" s="42" t="inlineStr">
-        <is>
-          <t>Name (print)</t>
-        </is>
-      </c>
-      <c r="D42" s="55" t="n"/>
+      <c r="C42" s="66" t="inlineStr">
+        <is>
+          <t>To accept the work, prices and terms above, sign below and return it with the deposit.</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="n"/>
       <c r="E42" s="13" t="n"/>
       <c r="F42" s="10" t="n"/>
-      <c r="G42" s="64" t="inlineStr">
+      <c r="G42" s="67" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H42" s="65" t="n"/>
-      <c r="I42" s="65" t="n"/>
-      <c r="J42" s="66">
+      <c r="H42" s="68" t="n"/>
+      <c r="I42" s="68" t="n"/>
+      <c r="J42" s="69">
         <f>IF($J$39="","",$J$39+$J$40+$J$41)</f>
         <v/>
       </c>
@@ -5272,7 +5375,7 @@
       <c r="B43" s="10" t="n"/>
       <c r="C43" s="42" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Name (print)</t>
         </is>
       </c>
       <c r="D43" s="55" t="n"/>
@@ -5284,7 +5387,7 @@
       </c>
       <c r="H43" s="48" t="n"/>
       <c r="I43" s="48" t="n"/>
-      <c r="J43" s="62">
+      <c r="J43" s="63">
         <f>IF($J$42="","",ROUND($J$42*N($J$20),2))</f>
         <v/>
       </c>
@@ -5310,20 +5413,20 @@
       <c r="B44" s="10" t="n"/>
       <c r="C44" s="42" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="D44" s="55" t="n"/>
       <c r="E44" s="13" t="n"/>
       <c r="F44" s="10" t="n"/>
-      <c r="G44" s="67" t="inlineStr">
+      <c r="G44" s="70" t="inlineStr">
         <is>
           <t>Balance due</t>
         </is>
       </c>
       <c r="H44" s="48" t="n"/>
       <c r="I44" s="48" t="n"/>
-      <c r="J44" s="68">
+      <c r="J44" s="71">
         <f>IF($J$42="","",$J$42-$J$43)</f>
         <v/>
       </c>
@@ -5346,16 +5449,20 @@
     </row>
     <row r="45" ht="21" customHeight="1">
       <c r="A45" s="1" t="n"/>
-      <c r="B45" s="15" t="n"/>
-      <c r="C45" s="16" t="n"/>
-      <c r="D45" s="16" t="n"/>
-      <c r="E45" s="17" t="n"/>
-      <c r="F45" s="15" t="n"/>
-      <c r="G45" s="16" t="n"/>
-      <c r="H45" s="16" t="n"/>
-      <c r="I45" s="16" t="n"/>
-      <c r="J45" s="16" t="n"/>
-      <c r="K45" s="17" t="n"/>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="42" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D45" s="55" t="n"/>
+      <c r="E45" s="13" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="12" t="n"/>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="12" t="n"/>
+      <c r="K45" s="13" t="n"/>
       <c r="L45" s="1" t="n"/>
       <c r="M45" s="1" t="n"/>
       <c r="N45" s="1" t="n"/>
@@ -5372,22 +5479,18 @@
       <c r="Y45" s="1" t="n"/>
       <c r="Z45" s="1" t="n"/>
     </row>
-    <row r="46" ht="24" customHeight="1">
+    <row r="46" ht="21" customHeight="1">
       <c r="A46" s="1" t="n"/>
-      <c r="B46" s="1" t="n"/>
-      <c r="C46" s="69" t="inlineStr">
-        <is>
-          <t>Sample estimate form to adapt. Have a local attorney review your terms before you use them with clients. Amounts are estimates for the work listed.</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="n"/>
-      <c r="E46" s="1" t="n"/>
-      <c r="F46" s="1" t="n"/>
-      <c r="G46" s="1" t="n"/>
-      <c r="H46" s="1" t="n"/>
-      <c r="I46" s="1" t="n"/>
-      <c r="J46" s="1" t="n"/>
-      <c r="K46" s="1" t="n"/>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="16" t="n"/>
+      <c r="D46" s="16" t="n"/>
+      <c r="E46" s="17" t="n"/>
+      <c r="F46" s="15" t="n"/>
+      <c r="G46" s="16" t="n"/>
+      <c r="H46" s="16" t="n"/>
+      <c r="I46" s="16" t="n"/>
+      <c r="J46" s="16" t="n"/>
+      <c r="K46" s="17" t="n"/>
       <c r="L46" s="1" t="n"/>
       <c r="M46" s="1" t="n"/>
       <c r="N46" s="1" t="n"/>
@@ -5404,10 +5507,14 @@
       <c r="Y46" s="1" t="n"/>
       <c r="Z46" s="1" t="n"/>
     </row>
-    <row r="47" ht="12" customHeight="1">
+    <row r="47" ht="24" customHeight="1">
       <c r="A47" s="1" t="n"/>
       <c r="B47" s="1" t="n"/>
-      <c r="C47" s="1" t="n"/>
+      <c r="C47" s="72" t="inlineStr">
+        <is>
+          <t>Sample estimate form to adapt. Have a local attorney review your terms before you use them with clients. Amounts are estimates for the work listed.</t>
+        </is>
+      </c>
       <c r="D47" s="1" t="n"/>
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="n"/>
@@ -5432,7 +5539,7 @@
       <c r="Y47" s="1" t="n"/>
       <c r="Z47" s="1" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" ht="12" customHeight="1">
       <c r="A48" s="1" t="n"/>
       <c r="B48" s="1" t="n"/>
       <c r="C48" s="1" t="n"/>
@@ -6524,20 +6631,49 @@
       <c r="Y86" s="1" t="n"/>
       <c r="Z86" s="1" t="n"/>
     </row>
+    <row r="87">
+      <c r="A87" s="1" t="n"/>
+      <c r="B87" s="1" t="n"/>
+      <c r="C87" s="1" t="n"/>
+      <c r="D87" s="1" t="n"/>
+      <c r="E87" s="1" t="n"/>
+      <c r="F87" s="1" t="n"/>
+      <c r="G87" s="1" t="n"/>
+      <c r="H87" s="1" t="n"/>
+      <c r="I87" s="1" t="n"/>
+      <c r="J87" s="1" t="n"/>
+      <c r="K87" s="1" t="n"/>
+      <c r="L87" s="1" t="n"/>
+      <c r="M87" s="1" t="n"/>
+      <c r="N87" s="1" t="n"/>
+      <c r="O87" s="1" t="n"/>
+      <c r="P87" s="1" t="n"/>
+      <c r="Q87" s="1" t="n"/>
+      <c r="R87" s="1" t="n"/>
+      <c r="S87" s="1" t="n"/>
+      <c r="T87" s="1" t="n"/>
+      <c r="U87" s="1" t="n"/>
+      <c r="V87" s="1" t="n"/>
+      <c r="W87" s="1" t="n"/>
+      <c r="X87" s="1" t="n"/>
+      <c r="Y87" s="1" t="n"/>
+      <c r="Z87" s="1" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C24:J24"/>
+    <mergeCell ref="C42:D42"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="C25:J25"/>
-    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C47:J47"/>
     <mergeCell ref="G12:J12"/>
     <mergeCell ref="I4:K4"/>
+    <mergeCell ref="C40:C41"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="G8:J8"/>
-    <mergeCell ref="C46:J46"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="C17:D17"/>
@@ -6546,6 +6682,7 @@
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="C7:D7"/>
+    <mergeCell ref="D40:D41"/>
   </mergeCells>
   <dataValidations count="19">
     <dataValidation sqref="D13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 60 characters." promptTitle="Business name" prompt="Your business name as customers know it, for example Brightside Exterior Cleaning." type="textLength" errorStyle="stop" operator="between">
@@ -6953,7 +7090,7 @@
     <row r="8" ht="24.8" customHeight="1">
       <c r="A8" s="1" t="n"/>
       <c r="B8" s="10" t="n"/>
-      <c r="C8" s="70" t="inlineStr">
+      <c r="C8" s="73" t="inlineStr">
         <is>
           <t>Pressure washing price calculator</t>
         </is>
@@ -6985,7 +7122,7 @@
     <row r="9" ht="24.8" customHeight="1">
       <c r="A9" s="1" t="n"/>
       <c r="B9" s="10" t="n"/>
-      <c r="C9" s="70" t="inlineStr">
+      <c r="C9" s="73" t="inlineStr">
         <is>
           <t>House cleaning price calculator</t>
         </is>
@@ -7017,7 +7154,7 @@
     <row r="10" ht="24.8" customHeight="1">
       <c r="A10" s="1" t="n"/>
       <c r="B10" s="10" t="n"/>
-      <c r="C10" s="70" t="inlineStr">
+      <c r="C10" s="73" t="inlineStr">
         <is>
           <t>Lawn care price calculator</t>
         </is>
@@ -7049,7 +7186,7 @@
     <row r="11" ht="24.8" customHeight="1">
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="10" t="n"/>
-      <c r="C11" s="70" t="inlineStr">
+      <c r="C11" s="73" t="inlineStr">
         <is>
           <t>Price increase calculator</t>
         </is>

</xml_diff>

<commit_message>
Templates design round 2 fixes; newest calculators join their clusters; launch record, handoff
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0122otiWoh8gJECjGVg2FuAQ
</commit_message>
<xml_diff>
--- a/docs/downloads/job-estimate-template.xlsx
+++ b/docs/downloads/job-estimate-template.xlsx
@@ -22,7 +22,7 @@
     <definedName name="DepositRate">'Estimate'!$J$20</definedName>
     <definedName name="PaymentTerms">'Estimate'!$D$40</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Start Here'!$A$1:$G$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Estimate'!$A$1:$L$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Estimate'!$A$1:$L$50</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Terms'!$A$1:$G$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -610,7 +610,7 @@
       <alignment horizontal="right" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="15" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="left" vertical="center" shrinkToFit="1" indent="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -626,7 +626,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+      <alignment horizontal="right" vertical="center" shrinkToFit="1" indent="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -643,13 +643,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="9" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+      <alignment horizontal="right" vertical="center" shrinkToFit="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+      <alignment horizontal="right" vertical="center" shrinkToFit="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -1067,7 +1067,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Job Estimate Template</t>
+          <t>Job estimate template</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -3790,7 +3790,7 @@
   <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8 ProofNotFluff&amp;R&amp;"Arial"&amp;8 Job Estimate Template</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8 ProofNotFluff&amp;R&amp;"Arial"&amp;8 Job estimate template</oddHeader>
     <oddFooter>&amp;L&amp;"Arial"&amp;8 Sample form. Estimates only, not legal or tax advice. See the Terms tab.&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -3810,19 +3810,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z87"/>
+  <dimension ref="A1:Z89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="2" customWidth="1" min="5" max="5"/>
     <col width="2" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="2" customWidth="1" min="11" max="11"/>
     <col width="3" customWidth="1" min="12" max="12"/>
   </cols>
@@ -4215,7 +4215,7 @@
       <c r="Y10" s="1" t="n"/>
       <c r="Z10" s="1" t="n"/>
     </row>
-    <row r="11" ht="21" customHeight="1">
+    <row r="11" ht="10" customHeight="1">
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="8" t="n"/>
@@ -4756,7 +4756,7 @@
       <c r="Y25" s="1" t="n"/>
       <c r="Z25" s="1" t="n"/>
     </row>
-    <row r="26" ht="8" customHeight="1">
+    <row r="26" ht="6" customHeight="1">
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="12" t="n"/>
@@ -4784,7 +4784,7 @@
       <c r="Y26" s="1" t="n"/>
       <c r="Z26" s="1" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="20" customHeight="1">
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="10" t="n"/>
       <c r="C27" s="54" t="inlineStr">
@@ -5188,7 +5188,7 @@
       <c r="Y37" s="1" t="n"/>
       <c r="Z37" s="1" t="n"/>
     </row>
-    <row r="38" ht="21" customHeight="1">
+    <row r="38" ht="10" customHeight="1">
       <c r="A38" s="1" t="n"/>
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="8" t="n"/>
@@ -5373,12 +5373,8 @@
     <row r="43" ht="21" customHeight="1">
       <c r="A43" s="1" t="n"/>
       <c r="B43" s="10" t="n"/>
-      <c r="C43" s="42" t="inlineStr">
-        <is>
-          <t>Name (print)</t>
-        </is>
-      </c>
-      <c r="D43" s="55" t="n"/>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
       <c r="E43" s="13" t="n"/>
       <c r="F43" s="10" t="n"/>
       <c r="G43" s="47">
@@ -5411,12 +5407,8 @@
     <row r="44" ht="21" customHeight="1">
       <c r="A44" s="1" t="n"/>
       <c r="B44" s="10" t="n"/>
-      <c r="C44" s="42" t="inlineStr">
-        <is>
-          <t>Signature</t>
-        </is>
-      </c>
-      <c r="D44" s="55" t="n"/>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
       <c r="E44" s="13" t="n"/>
       <c r="F44" s="10" t="n"/>
       <c r="G44" s="70" t="inlineStr">
@@ -5452,7 +5444,7 @@
       <c r="B45" s="10" t="n"/>
       <c r="C45" s="42" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Name (print)</t>
         </is>
       </c>
       <c r="D45" s="55" t="n"/>
@@ -5481,16 +5473,20 @@
     </row>
     <row r="46" ht="21" customHeight="1">
       <c r="A46" s="1" t="n"/>
-      <c r="B46" s="15" t="n"/>
-      <c r="C46" s="16" t="n"/>
-      <c r="D46" s="16" t="n"/>
-      <c r="E46" s="17" t="n"/>
-      <c r="F46" s="15" t="n"/>
-      <c r="G46" s="16" t="n"/>
-      <c r="H46" s="16" t="n"/>
-      <c r="I46" s="16" t="n"/>
-      <c r="J46" s="16" t="n"/>
-      <c r="K46" s="17" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="42" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="D46" s="55" t="n"/>
+      <c r="E46" s="13" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="12" t="n"/>
+      <c r="H46" s="12" t="n"/>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="12" t="n"/>
+      <c r="K46" s="13" t="n"/>
       <c r="L46" s="1" t="n"/>
       <c r="M46" s="1" t="n"/>
       <c r="N46" s="1" t="n"/>
@@ -5507,22 +5503,22 @@
       <c r="Y46" s="1" t="n"/>
       <c r="Z46" s="1" t="n"/>
     </row>
-    <row r="47" ht="24" customHeight="1">
+    <row r="47" ht="21" customHeight="1">
       <c r="A47" s="1" t="n"/>
-      <c r="B47" s="1" t="n"/>
-      <c r="C47" s="72" t="inlineStr">
-        <is>
-          <t>Sample estimate form to adapt. Have a local attorney review your terms before you use them with clients. Amounts are estimates for the work listed.</t>
-        </is>
-      </c>
-      <c r="D47" s="1" t="n"/>
-      <c r="E47" s="1" t="n"/>
-      <c r="F47" s="1" t="n"/>
-      <c r="G47" s="1" t="n"/>
-      <c r="H47" s="1" t="n"/>
-      <c r="I47" s="1" t="n"/>
-      <c r="J47" s="1" t="n"/>
-      <c r="K47" s="1" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="42" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D47" s="55" t="n"/>
+      <c r="E47" s="13" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="12" t="n"/>
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="12" t="n"/>
+      <c r="K47" s="13" t="n"/>
       <c r="L47" s="1" t="n"/>
       <c r="M47" s="1" t="n"/>
       <c r="N47" s="1" t="n"/>
@@ -5539,18 +5535,18 @@
       <c r="Y47" s="1" t="n"/>
       <c r="Z47" s="1" t="n"/>
     </row>
-    <row r="48" ht="12" customHeight="1">
+    <row r="48" ht="21" customHeight="1">
       <c r="A48" s="1" t="n"/>
-      <c r="B48" s="1" t="n"/>
-      <c r="C48" s="1" t="n"/>
-      <c r="D48" s="1" t="n"/>
-      <c r="E48" s="1" t="n"/>
-      <c r="F48" s="1" t="n"/>
-      <c r="G48" s="1" t="n"/>
-      <c r="H48" s="1" t="n"/>
-      <c r="I48" s="1" t="n"/>
-      <c r="J48" s="1" t="n"/>
-      <c r="K48" s="1" t="n"/>
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="16" t="n"/>
+      <c r="D48" s="16" t="n"/>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="16" t="n"/>
+      <c r="H48" s="16" t="n"/>
+      <c r="I48" s="16" t="n"/>
+      <c r="J48" s="16" t="n"/>
+      <c r="K48" s="17" t="n"/>
       <c r="L48" s="1" t="n"/>
       <c r="M48" s="1" t="n"/>
       <c r="N48" s="1" t="n"/>
@@ -5567,10 +5563,14 @@
       <c r="Y48" s="1" t="n"/>
       <c r="Z48" s="1" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="24" customHeight="1">
       <c r="A49" s="1" t="n"/>
       <c r="B49" s="1" t="n"/>
-      <c r="C49" s="1" t="n"/>
+      <c r="C49" s="72" t="inlineStr">
+        <is>
+          <t>Sample estimate form to adapt. Have a local attorney review your terms before you use them with clients. Amounts are estimates for the work listed.</t>
+        </is>
+      </c>
       <c r="D49" s="1" t="n"/>
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="n"/>
@@ -5595,7 +5595,7 @@
       <c r="Y49" s="1" t="n"/>
       <c r="Z49" s="1" t="n"/>
     </row>
-    <row r="50">
+    <row r="50" ht="12" customHeight="1">
       <c r="A50" s="1" t="n"/>
       <c r="B50" s="1" t="n"/>
       <c r="C50" s="1" t="n"/>
@@ -6659,16 +6659,71 @@
       <c r="Y87" s="1" t="n"/>
       <c r="Z87" s="1" t="n"/>
     </row>
+    <row r="88">
+      <c r="A88" s="1" t="n"/>
+      <c r="B88" s="1" t="n"/>
+      <c r="C88" s="1" t="n"/>
+      <c r="D88" s="1" t="n"/>
+      <c r="E88" s="1" t="n"/>
+      <c r="F88" s="1" t="n"/>
+      <c r="G88" s="1" t="n"/>
+      <c r="H88" s="1" t="n"/>
+      <c r="I88" s="1" t="n"/>
+      <c r="J88" s="1" t="n"/>
+      <c r="K88" s="1" t="n"/>
+      <c r="L88" s="1" t="n"/>
+      <c r="M88" s="1" t="n"/>
+      <c r="N88" s="1" t="n"/>
+      <c r="O88" s="1" t="n"/>
+      <c r="P88" s="1" t="n"/>
+      <c r="Q88" s="1" t="n"/>
+      <c r="R88" s="1" t="n"/>
+      <c r="S88" s="1" t="n"/>
+      <c r="T88" s="1" t="n"/>
+      <c r="U88" s="1" t="n"/>
+      <c r="V88" s="1" t="n"/>
+      <c r="W88" s="1" t="n"/>
+      <c r="X88" s="1" t="n"/>
+      <c r="Y88" s="1" t="n"/>
+      <c r="Z88" s="1" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n"/>
+      <c r="B89" s="1" t="n"/>
+      <c r="C89" s="1" t="n"/>
+      <c r="D89" s="1" t="n"/>
+      <c r="E89" s="1" t="n"/>
+      <c r="F89" s="1" t="n"/>
+      <c r="G89" s="1" t="n"/>
+      <c r="H89" s="1" t="n"/>
+      <c r="I89" s="1" t="n"/>
+      <c r="J89" s="1" t="n"/>
+      <c r="K89" s="1" t="n"/>
+      <c r="L89" s="1" t="n"/>
+      <c r="M89" s="1" t="n"/>
+      <c r="N89" s="1" t="n"/>
+      <c r="O89" s="1" t="n"/>
+      <c r="P89" s="1" t="n"/>
+      <c r="Q89" s="1" t="n"/>
+      <c r="R89" s="1" t="n"/>
+      <c r="S89" s="1" t="n"/>
+      <c r="T89" s="1" t="n"/>
+      <c r="U89" s="1" t="n"/>
+      <c r="V89" s="1" t="n"/>
+      <c r="W89" s="1" t="n"/>
+      <c r="X89" s="1" t="n"/>
+      <c r="Y89" s="1" t="n"/>
+      <c r="Z89" s="1" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="21">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C24:J24"/>
-    <mergeCell ref="C42:D42"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="C25:J25"/>
-    <mergeCell ref="C47:J47"/>
     <mergeCell ref="G12:J12"/>
+    <mergeCell ref="D40:D41"/>
     <mergeCell ref="I4:K4"/>
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C12:D12"/>
@@ -6680,9 +6735,10 @@
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="G6:J6"/>
+    <mergeCell ref="C42:D43"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="C49:J49"/>
   </mergeCells>
   <dataValidations count="19">
     <dataValidation sqref="D13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 60 characters." promptTitle="Business name" prompt="Your business name as customers know it, for example Brightside Exterior Cleaning." type="textLength" errorStyle="stop" operator="between">
@@ -6737,25 +6793,25 @@
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="C28:C35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 40 characters." promptTitle="Item" prompt="A short name, for example Driveway." type="textLength" errorStyle="stop" operator="between">
+    <dataValidation sqref="C28:C35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 20 characters, so it prints in full." promptTitle="Item" prompt="A short name, up to 20 characters, for example Driveway." type="textLength" errorStyle="stop" operator="between">
       <formula1>0</formula1>
-      <formula2>40</formula2>
+      <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="D28:D35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 80 characters." promptTitle="Description" prompt="What the work covers, for example 2-car concrete driveway, surface clean." type="textLength" errorStyle="stop" operator="between">
+    <dataValidation sqref="D28:D35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 36 characters, so it prints in full." promptTitle="Description" prompt="What the work covers, up to 36 characters, for example 2-car concrete, surface clean." type="textLength" errorStyle="stop" operator="between">
       <formula1>0</formula1>
-      <formula2>80</formula2>
+      <formula2>36</formula2>
     </dataValidation>
-    <dataValidation sqref="G28:G35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Type a quantity of 0 or more." promptTitle="Qty" prompt="How many: 1 job, 3 hours, 450 sq ft. A number of 0 or more." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="G28:G35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Type a quantity from 0 to 9,999." promptTitle="Qty" prompt="How many: 1 job, 3 hours, 450 sq ft. A number from 0 to 9,999." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
-      <formula2>1000000</formula2>
+      <formula2>9999</formula2>
     </dataValidation>
     <dataValidation sqref="H28:H35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 12 characters." promptTitle="Unit" prompt="What one is, for example job, hour, visit or sq ft. Optional." type="textLength" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>12</formula2>
     </dataValidation>
-    <dataValidation sqref="I28:I35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Type a price in dollars." promptTitle="Rate" prompt="Price for one unit, in dollars, for example 200. A credit can be negative." type="decimal" errorStyle="stop" operator="between">
-      <formula1>-1000000</formula1>
-      <formula2>1000000</formula2>
+    <dataValidation sqref="I28:I35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Type a rate from -$99,999 to $99,999." promptTitle="Rate" prompt="Price for one unit, in dollars, for example 200. A credit can be negative. From -$99,999 to $99,999." type="decimal" errorStyle="stop" operator="between">
+      <formula1>-99999</formula1>
+      <formula2>99999</formula2>
     </dataValidation>
     <dataValidation sqref="D40" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Check this cell" error="Up to 60 characters." promptTitle="Payment terms" prompt="One short line, for example Balance due when the job is done." type="textLength" errorStyle="stop" operator="between">
       <formula1>0</formula1>
@@ -6766,7 +6822,7 @@
   <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8 ProofNotFluff&amp;R&amp;"Arial"&amp;8 Job Estimate Template</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8 ProofNotFluff&amp;R&amp;"Arial"&amp;8 Job estimate template</oddHeader>
     <oddFooter>&amp;L&amp;"Arial"&amp;8 Sample form. Estimates only, not legal or tax advice. See the Terms tab.&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -6967,7 +7023,7 @@
       <c r="A4" s="1" t="n"/>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Job Estimate Template, version 1. Read this before you rely on a number.</t>
+          <t>Job estimate template, version 1. Read this before you rely on a number.</t>
         </is>
       </c>
       <c r="C4" s="1" t="n"/>
@@ -9042,7 +9098,7 @@
   <pageMargins left="0.5" right="0.5" top="0.7" bottom="0.7" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8 ProofNotFluff&amp;R&amp;"Arial"&amp;8 Job Estimate Template</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8 ProofNotFluff&amp;R&amp;"Arial"&amp;8 Job estimate template</oddHeader>
     <oddFooter>&amp;L&amp;"Arial"&amp;8 Estimates only. Not professional advice. See the Terms tab.&amp;R&amp;"Arial"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>